<commit_message>
atualizando ados sorteios Excel
</commit_message>
<xml_diff>
--- a/LoteriasExcel/Lotomania_edt.xlsx
+++ b/LoteriasExcel/Lotomania_edt.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Dell\Dropbox\! 000 ByPass\Pessoal\99_Loterias\0 - Loterias-Inteligentes\LoteriasExcel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1106539D-26CE-42AE-9812-59661B744A1B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B74069DC-5AEB-4C9C-ACC1-D13D15F69EF0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="58095" yWindow="3090" windowWidth="25950" windowHeight="17475" tabRatio="876" xr2:uid="{2663372B-AA50-4721-AD6B-5F0B8186ACF5}"/>
+    <workbookView xWindow="57585" yWindow="1770" windowWidth="19485" windowHeight="18465" tabRatio="876" xr2:uid="{2663372B-AA50-4721-AD6B-5F0B8186ACF5}"/>
   </bookViews>
   <sheets>
     <sheet name="LOTOMANIA" sheetId="6" r:id="rId1"/>
@@ -473,16 +473,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7C50A779-EE49-4F4E-A3D3-22C3D200C502}">
-  <dimension ref="A1:V385"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <dimension ref="A1:V401"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="22" max="22" width="13.07421875" customWidth="1"/>
-    <col min="23" max="23" width="19.07421875" customWidth="1"/>
+    <col min="22" max="22" width="13.06640625" customWidth="1"/>
+    <col min="23" max="23" width="19.06640625" customWidth="1"/>
     <col min="24" max="24" width="13" customWidth="1"/>
-    <col min="25" max="25" width="9.69140625" customWidth="1"/>
+    <col min="25" max="25" width="9.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -547,7 +547,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="2" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A2">
         <v>2508</v>
       </c>
@@ -612,7 +612,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="3" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A3">
         <v>2509</v>
       </c>
@@ -677,7 +677,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="4" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A4">
         <v>2510</v>
       </c>
@@ -742,7 +742,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="5" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A5">
         <v>2511</v>
       </c>
@@ -807,7 +807,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="6" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A6">
         <v>2512</v>
       </c>
@@ -872,7 +872,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="7" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A7">
         <v>2513</v>
       </c>
@@ -937,7 +937,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="8" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A8">
         <v>2514</v>
       </c>
@@ -1002,7 +1002,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="9" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A9">
         <v>2515</v>
       </c>
@@ -1067,7 +1067,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="10" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A10">
         <v>2516</v>
       </c>
@@ -1132,7 +1132,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="11" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A11">
         <v>2517</v>
       </c>
@@ -1197,7 +1197,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="12" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A12">
         <v>2518</v>
       </c>
@@ -1262,7 +1262,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="13" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A13">
         <v>2519</v>
       </c>
@@ -1327,7 +1327,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="14" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A14">
         <v>2520</v>
       </c>
@@ -1392,7 +1392,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="15" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A15">
         <v>2521</v>
       </c>
@@ -1457,7 +1457,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="16" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A16">
         <v>2522</v>
       </c>
@@ -1522,7 +1522,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="17" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A17">
         <v>2523</v>
       </c>
@@ -1587,7 +1587,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="18" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A18">
         <v>2524</v>
       </c>
@@ -1652,7 +1652,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="19" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A19">
         <v>2525</v>
       </c>
@@ -1717,7 +1717,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="20" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A20">
         <v>2526</v>
       </c>
@@ -1782,7 +1782,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="21" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="21" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A21">
         <v>2527</v>
       </c>
@@ -1847,7 +1847,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="22" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="22" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A22">
         <v>2528</v>
       </c>
@@ -1912,7 +1912,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="23" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="23" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A23">
         <v>2529</v>
       </c>
@@ -1977,7 +1977,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="24" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="24" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A24">
         <v>2530</v>
       </c>
@@ -2042,7 +2042,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="25" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="25" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A25">
         <v>2531</v>
       </c>
@@ -2107,7 +2107,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="26" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="26" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A26">
         <v>2532</v>
       </c>
@@ -2172,7 +2172,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="27" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="27" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A27">
         <v>2533</v>
       </c>
@@ -2237,7 +2237,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="28" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="28" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A28">
         <v>2534</v>
       </c>
@@ -2302,7 +2302,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="29" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="29" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A29">
         <v>2535</v>
       </c>
@@ -2367,7 +2367,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="30" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="30" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A30">
         <v>2536</v>
       </c>
@@ -2432,7 +2432,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="31" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="31" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A31">
         <v>2537</v>
       </c>
@@ -2497,7 +2497,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="32" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="32" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A32">
         <v>2538</v>
       </c>
@@ -2562,7 +2562,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="33" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="33" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A33">
         <v>2539</v>
       </c>
@@ -2627,7 +2627,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="34" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="34" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A34">
         <v>2540</v>
       </c>
@@ -2692,7 +2692,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="35" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="35" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A35">
         <v>2541</v>
       </c>
@@ -2757,7 +2757,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="36" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="36" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A36">
         <v>2542</v>
       </c>
@@ -2822,7 +2822,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="37" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="37" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A37">
         <v>2543</v>
       </c>
@@ -2887,7 +2887,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="38" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="38" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A38">
         <v>2544</v>
       </c>
@@ -2952,7 +2952,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="39" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="39" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A39">
         <v>2545</v>
       </c>
@@ -3017,7 +3017,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="40" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="40" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A40">
         <v>2546</v>
       </c>
@@ -3082,7 +3082,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="41" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="41" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A41">
         <v>2547</v>
       </c>
@@ -3147,7 +3147,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="42" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="42" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A42">
         <v>2548</v>
       </c>
@@ -3212,7 +3212,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="43" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="43" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A43">
         <v>2549</v>
       </c>
@@ -3277,7 +3277,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="44" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="44" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A44">
         <v>2550</v>
       </c>
@@ -3342,7 +3342,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="45" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="45" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A45">
         <v>2551</v>
       </c>
@@ -3407,7 +3407,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="46" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="46" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A46">
         <v>2552</v>
       </c>
@@ -3472,7 +3472,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="47" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="47" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A47">
         <v>2553</v>
       </c>
@@ -3537,7 +3537,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="48" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="48" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A48">
         <v>2554</v>
       </c>
@@ -3602,7 +3602,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="49" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="49" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A49">
         <v>2555</v>
       </c>
@@ -3667,7 +3667,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="50" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="50" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A50">
         <v>2556</v>
       </c>
@@ -3732,7 +3732,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="51" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="51" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A51">
         <v>2557</v>
       </c>
@@ -3797,7 +3797,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="52" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="52" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A52">
         <v>2558</v>
       </c>
@@ -3862,7 +3862,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="53" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="53" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A53">
         <v>2559</v>
       </c>
@@ -3927,7 +3927,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="54" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="54" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A54">
         <v>2560</v>
       </c>
@@ -3992,7 +3992,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="55" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="55" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A55">
         <v>2561</v>
       </c>
@@ -4057,7 +4057,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="56" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="56" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A56">
         <v>2562</v>
       </c>
@@ -4122,7 +4122,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="57" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="57" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A57">
         <v>2563</v>
       </c>
@@ -4187,7 +4187,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="58" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="58" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A58">
         <v>2564</v>
       </c>
@@ -4252,7 +4252,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="59" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="59" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A59">
         <v>2565</v>
       </c>
@@ -4317,7 +4317,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="60" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="60" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A60">
         <v>2566</v>
       </c>
@@ -4382,7 +4382,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="61" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="61" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A61">
         <v>2567</v>
       </c>
@@ -4447,7 +4447,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="62" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="62" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A62">
         <v>2568</v>
       </c>
@@ -4512,7 +4512,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="63" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="63" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A63">
         <v>2569</v>
       </c>
@@ -4577,7 +4577,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="64" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="64" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A64">
         <v>2570</v>
       </c>
@@ -4642,7 +4642,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="65" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="65" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A65">
         <v>2571</v>
       </c>
@@ -4707,7 +4707,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="66" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="66" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A66">
         <v>2572</v>
       </c>
@@ -4772,7 +4772,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="67" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="67" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A67">
         <v>2573</v>
       </c>
@@ -4837,7 +4837,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="68" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="68" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A68">
         <v>2574</v>
       </c>
@@ -4902,7 +4902,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="69" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="69" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A69">
         <v>2575</v>
       </c>
@@ -4967,7 +4967,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="70" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="70" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A70">
         <v>2576</v>
       </c>
@@ -5032,7 +5032,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="71" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="71" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A71">
         <v>2577</v>
       </c>
@@ -5097,7 +5097,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="72" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="72" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A72">
         <v>2578</v>
       </c>
@@ -5162,7 +5162,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="73" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="73" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A73">
         <v>2579</v>
       </c>
@@ -5227,7 +5227,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="74" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="74" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A74">
         <v>2580</v>
       </c>
@@ -5292,7 +5292,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="75" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="75" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A75">
         <v>2581</v>
       </c>
@@ -5357,7 +5357,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="76" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="76" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A76">
         <v>2582</v>
       </c>
@@ -5422,7 +5422,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="77" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="77" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A77">
         <v>2583</v>
       </c>
@@ -5487,7 +5487,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="78" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="78" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A78">
         <v>2584</v>
       </c>
@@ -5552,7 +5552,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="79" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="79" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A79">
         <v>2585</v>
       </c>
@@ -5617,7 +5617,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="80" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="80" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A80">
         <v>2586</v>
       </c>
@@ -5682,7 +5682,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="81" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="81" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A81">
         <v>2587</v>
       </c>
@@ -5747,7 +5747,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="82" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="82" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A82">
         <v>2588</v>
       </c>
@@ -5812,7 +5812,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="83" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="83" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A83">
         <v>2589</v>
       </c>
@@ -5877,7 +5877,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="84" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="84" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A84">
         <v>2590</v>
       </c>
@@ -5942,7 +5942,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="85" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="85" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A85">
         <v>2591</v>
       </c>
@@ -6007,7 +6007,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="86" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="86" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A86">
         <v>2592</v>
       </c>
@@ -6072,7 +6072,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="87" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="87" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A87">
         <v>2593</v>
       </c>
@@ -6137,7 +6137,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="88" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="88" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A88">
         <v>2594</v>
       </c>
@@ -6202,7 +6202,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="89" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="89" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A89">
         <v>2595</v>
       </c>
@@ -6267,7 +6267,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="90" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="90" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A90">
         <v>2596</v>
       </c>
@@ -6332,7 +6332,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="91" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="91" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A91">
         <v>2597</v>
       </c>
@@ -6397,7 +6397,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="92" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="92" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A92">
         <v>2598</v>
       </c>
@@ -6462,7 +6462,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="93" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="93" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A93">
         <v>2599</v>
       </c>
@@ -6527,7 +6527,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="94" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="94" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A94">
         <v>2600</v>
       </c>
@@ -6592,7 +6592,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="95" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="95" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A95">
         <v>2601</v>
       </c>
@@ -6657,7 +6657,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="96" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="96" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A96">
         <v>2602</v>
       </c>
@@ -6722,7 +6722,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="97" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="97" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A97">
         <v>2603</v>
       </c>
@@ -6787,7 +6787,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="98" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="98" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A98">
         <v>2604</v>
       </c>
@@ -6852,7 +6852,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="99" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="99" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A99">
         <v>2605</v>
       </c>
@@ -6917,7 +6917,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="100" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="100" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A100">
         <v>2606</v>
       </c>
@@ -6982,7 +6982,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="101" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="101" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A101">
         <v>2607</v>
       </c>
@@ -7047,7 +7047,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="102" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="102" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A102">
         <v>2608</v>
       </c>
@@ -7112,7 +7112,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="103" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="103" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A103">
         <v>2609</v>
       </c>
@@ -7177,7 +7177,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="104" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="104" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A104">
         <v>2610</v>
       </c>
@@ -7242,7 +7242,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="105" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="105" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A105">
         <v>2611</v>
       </c>
@@ -7307,7 +7307,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="106" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="106" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A106">
         <v>2612</v>
       </c>
@@ -7372,7 +7372,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="107" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="107" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A107">
         <v>2613</v>
       </c>
@@ -7437,7 +7437,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="108" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="108" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A108">
         <v>2614</v>
       </c>
@@ -7502,7 +7502,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="109" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="109" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A109">
         <v>2615</v>
       </c>
@@ -7567,7 +7567,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="110" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="110" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A110">
         <v>2616</v>
       </c>
@@ -7632,7 +7632,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="111" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="111" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A111">
         <v>2617</v>
       </c>
@@ -7697,7 +7697,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="112" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="112" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A112">
         <v>2618</v>
       </c>
@@ -7762,7 +7762,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="113" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="113" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A113">
         <v>2619</v>
       </c>
@@ -7827,7 +7827,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="114" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="114" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A114">
         <v>2620</v>
       </c>
@@ -7892,7 +7892,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="115" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="115" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A115">
         <v>2621</v>
       </c>
@@ -7957,7 +7957,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="116" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="116" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A116">
         <v>2622</v>
       </c>
@@ -8022,7 +8022,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="117" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="117" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A117">
         <v>2623</v>
       </c>
@@ -8087,7 +8087,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="118" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="118" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A118">
         <v>2624</v>
       </c>
@@ -8152,7 +8152,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="119" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="119" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A119">
         <v>2625</v>
       </c>
@@ -8217,7 +8217,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="120" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="120" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A120">
         <v>2626</v>
       </c>
@@ -8282,7 +8282,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="121" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="121" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A121">
         <v>2627</v>
       </c>
@@ -8347,7 +8347,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="122" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="122" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A122">
         <v>2628</v>
       </c>
@@ -8412,7 +8412,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="123" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="123" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A123">
         <v>2629</v>
       </c>
@@ -8477,7 +8477,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="124" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="124" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A124">
         <v>2630</v>
       </c>
@@ -8542,7 +8542,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="125" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="125" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A125">
         <v>2631</v>
       </c>
@@ -8607,7 +8607,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="126" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="126" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A126">
         <v>2632</v>
       </c>
@@ -8672,7 +8672,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="127" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="127" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A127">
         <v>2633</v>
       </c>
@@ -8737,7 +8737,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="128" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="128" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A128">
         <v>2634</v>
       </c>
@@ -8802,7 +8802,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="129" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="129" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A129">
         <v>2635</v>
       </c>
@@ -8867,7 +8867,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="130" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="130" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A130">
         <v>2636</v>
       </c>
@@ -8932,7 +8932,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="131" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="131" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A131">
         <v>2637</v>
       </c>
@@ -8997,7 +8997,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="132" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="132" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A132">
         <v>2638</v>
       </c>
@@ -9062,7 +9062,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="133" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="133" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A133">
         <v>2639</v>
       </c>
@@ -9127,7 +9127,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="134" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="134" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A134">
         <v>2640</v>
       </c>
@@ -9192,7 +9192,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="135" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="135" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A135">
         <v>2641</v>
       </c>
@@ -9257,7 +9257,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="136" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="136" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A136">
         <v>2642</v>
       </c>
@@ -9322,7 +9322,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="137" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="137" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A137">
         <v>2643</v>
       </c>
@@ -9387,7 +9387,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="138" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="138" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A138">
         <v>2644</v>
       </c>
@@ -9452,7 +9452,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="139" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="139" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A139">
         <v>2645</v>
       </c>
@@ -9517,7 +9517,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="140" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="140" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A140">
         <v>2646</v>
       </c>
@@ -9582,7 +9582,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="141" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="141" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A141">
         <v>2647</v>
       </c>
@@ -9647,7 +9647,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="142" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="142" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A142">
         <v>2648</v>
       </c>
@@ -9712,7 +9712,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="143" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="143" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A143">
         <v>2649</v>
       </c>
@@ -9777,7 +9777,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="144" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="144" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A144">
         <v>2650</v>
       </c>
@@ -9842,7 +9842,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="145" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="145" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A145">
         <v>2651</v>
       </c>
@@ -9907,7 +9907,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="146" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="146" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A146">
         <v>2652</v>
       </c>
@@ -9972,7 +9972,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="147" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="147" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A147">
         <v>2653</v>
       </c>
@@ -10037,7 +10037,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="148" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="148" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A148">
         <v>2654</v>
       </c>
@@ -10102,7 +10102,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="149" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="149" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A149">
         <v>2655</v>
       </c>
@@ -10167,7 +10167,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="150" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="150" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A150">
         <v>2656</v>
       </c>
@@ -10232,7 +10232,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="151" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="151" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A151">
         <v>2657</v>
       </c>
@@ -10297,7 +10297,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="152" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="152" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A152">
         <v>2658</v>
       </c>
@@ -10362,7 +10362,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="153" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="153" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A153">
         <v>2659</v>
       </c>
@@ -10427,7 +10427,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="154" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="154" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A154">
         <v>2660</v>
       </c>
@@ -10492,7 +10492,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="155" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="155" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A155">
         <v>2661</v>
       </c>
@@ -10557,7 +10557,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="156" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="156" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A156">
         <v>2662</v>
       </c>
@@ -10622,7 +10622,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="157" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="157" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A157">
         <v>2663</v>
       </c>
@@ -10687,7 +10687,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="158" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="158" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A158">
         <v>2664</v>
       </c>
@@ -10752,7 +10752,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="159" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="159" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A159">
         <v>2665</v>
       </c>
@@ -10817,7 +10817,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="160" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="160" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A160">
         <v>2666</v>
       </c>
@@ -10882,7 +10882,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="161" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="161" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A161">
         <v>2667</v>
       </c>
@@ -10947,7 +10947,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="162" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="162" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A162">
         <v>2668</v>
       </c>
@@ -11012,7 +11012,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="163" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="163" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A163">
         <v>2669</v>
       </c>
@@ -11077,7 +11077,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="164" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="164" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A164">
         <v>2670</v>
       </c>
@@ -11142,7 +11142,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="165" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="165" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A165">
         <v>2671</v>
       </c>
@@ -11207,7 +11207,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="166" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="166" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A166">
         <v>2672</v>
       </c>
@@ -11272,7 +11272,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="167" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="167" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A167">
         <v>2673</v>
       </c>
@@ -11337,7 +11337,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="168" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="168" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A168">
         <v>2674</v>
       </c>
@@ -11402,7 +11402,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="169" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="169" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A169">
         <v>2675</v>
       </c>
@@ -11467,7 +11467,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="170" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="170" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A170">
         <v>2676</v>
       </c>
@@ -11532,7 +11532,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="171" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="171" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A171">
         <v>2677</v>
       </c>
@@ -11597,7 +11597,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="172" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="172" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A172">
         <v>2678</v>
       </c>
@@ -11662,7 +11662,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="173" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="173" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A173">
         <v>2679</v>
       </c>
@@ -11727,7 +11727,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="174" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="174" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A174">
         <v>2680</v>
       </c>
@@ -11792,7 +11792,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="175" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="175" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A175">
         <v>2681</v>
       </c>
@@ -11857,7 +11857,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="176" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="176" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A176">
         <v>2682</v>
       </c>
@@ -11922,7 +11922,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="177" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="177" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A177">
         <v>2683</v>
       </c>
@@ -11987,7 +11987,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="178" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="178" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A178">
         <v>2684</v>
       </c>
@@ -12052,7 +12052,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="179" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="179" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A179">
         <v>2685</v>
       </c>
@@ -12117,7 +12117,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="180" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="180" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A180">
         <v>2686</v>
       </c>
@@ -12182,7 +12182,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="181" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="181" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A181">
         <v>2687</v>
       </c>
@@ -12247,7 +12247,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="182" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="182" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A182">
         <v>2688</v>
       </c>
@@ -12312,7 +12312,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="183" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="183" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A183">
         <v>2689</v>
       </c>
@@ -12377,7 +12377,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="184" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="184" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A184">
         <v>2690</v>
       </c>
@@ -12442,7 +12442,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="185" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="185" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A185">
         <v>2691</v>
       </c>
@@ -12507,7 +12507,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="186" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="186" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A186">
         <v>2692</v>
       </c>
@@ -12572,7 +12572,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="187" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="187" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A187">
         <v>2693</v>
       </c>
@@ -12637,7 +12637,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="188" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="188" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A188">
         <v>2694</v>
       </c>
@@ -12702,7 +12702,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="189" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="189" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A189">
         <v>2695</v>
       </c>
@@ -12767,7 +12767,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="190" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="190" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A190">
         <v>2696</v>
       </c>
@@ -12832,7 +12832,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="191" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="191" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A191">
         <v>2697</v>
       </c>
@@ -12897,7 +12897,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="192" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="192" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A192">
         <v>2698</v>
       </c>
@@ -12962,7 +12962,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="193" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="193" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A193">
         <v>2699</v>
       </c>
@@ -13027,7 +13027,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="194" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="194" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A194">
         <v>2700</v>
       </c>
@@ -13092,7 +13092,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="195" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="195" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A195">
         <v>2701</v>
       </c>
@@ -13157,7 +13157,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="196" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="196" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A196">
         <v>2702</v>
       </c>
@@ -13222,7 +13222,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="197" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="197" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A197">
         <v>2703</v>
       </c>
@@ -13287,7 +13287,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="198" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="198" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A198">
         <v>2704</v>
       </c>
@@ -13352,7 +13352,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="199" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="199" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A199">
         <v>2705</v>
       </c>
@@ -13417,7 +13417,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="200" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="200" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A200">
         <v>2706</v>
       </c>
@@ -13482,7 +13482,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="201" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="201" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A201">
         <v>2707</v>
       </c>
@@ -13547,7 +13547,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="202" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="202" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A202">
         <v>2708</v>
       </c>
@@ -13612,7 +13612,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="203" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="203" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A203">
         <v>2709</v>
       </c>
@@ -13677,7 +13677,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="204" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="204" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A204">
         <v>2710</v>
       </c>
@@ -13742,7 +13742,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="205" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="205" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A205">
         <v>2711</v>
       </c>
@@ -13807,7 +13807,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="206" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="206" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A206">
         <v>2712</v>
       </c>
@@ -13872,7 +13872,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="207" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="207" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A207">
         <v>2713</v>
       </c>
@@ -13937,7 +13937,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="208" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="208" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A208">
         <v>2714</v>
       </c>
@@ -14002,7 +14002,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="209" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="209" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A209">
         <v>2715</v>
       </c>
@@ -14067,7 +14067,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="210" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="210" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A210">
         <v>2716</v>
       </c>
@@ -14132,7 +14132,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="211" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="211" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A211">
         <v>2717</v>
       </c>
@@ -14197,7 +14197,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="212" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="212" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A212">
         <v>2718</v>
       </c>
@@ -14262,7 +14262,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="213" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="213" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A213">
         <v>2719</v>
       </c>
@@ -14327,7 +14327,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="214" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="214" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A214">
         <v>2720</v>
       </c>
@@ -14392,7 +14392,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="215" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="215" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A215">
         <v>2721</v>
       </c>
@@ -14457,7 +14457,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="216" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="216" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A216">
         <v>2722</v>
       </c>
@@ -14522,7 +14522,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="217" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="217" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A217">
         <v>2723</v>
       </c>
@@ -14587,7 +14587,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="218" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="218" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A218">
         <v>2724</v>
       </c>
@@ -14652,7 +14652,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="219" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="219" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A219">
         <v>2725</v>
       </c>
@@ -14717,7 +14717,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="220" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="220" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A220">
         <v>2726</v>
       </c>
@@ -14782,7 +14782,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="221" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="221" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A221">
         <v>2727</v>
       </c>
@@ -14847,7 +14847,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="222" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="222" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A222">
         <v>2728</v>
       </c>
@@ -14912,7 +14912,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="223" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="223" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A223">
         <v>2729</v>
       </c>
@@ -14977,7 +14977,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="224" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="224" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A224">
         <v>2730</v>
       </c>
@@ -15042,7 +15042,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="225" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="225" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A225">
         <v>2731</v>
       </c>
@@ -15107,7 +15107,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="226" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="226" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A226">
         <v>2732</v>
       </c>
@@ -15172,7 +15172,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="227" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="227" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A227">
         <v>2733</v>
       </c>
@@ -15237,7 +15237,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="228" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="228" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A228">
         <v>2734</v>
       </c>
@@ -15302,7 +15302,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="229" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="229" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A229">
         <v>2735</v>
       </c>
@@ -15367,7 +15367,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="230" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="230" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A230">
         <v>2736</v>
       </c>
@@ -15432,7 +15432,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="231" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="231" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A231">
         <v>2737</v>
       </c>
@@ -15497,7 +15497,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="232" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="232" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A232">
         <v>2738</v>
       </c>
@@ -15562,7 +15562,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="233" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="233" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A233">
         <v>2739</v>
       </c>
@@ -15627,7 +15627,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="234" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="234" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A234">
         <v>2740</v>
       </c>
@@ -15692,7 +15692,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="235" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="235" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A235">
         <v>2741</v>
       </c>
@@ -15757,7 +15757,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="236" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="236" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A236">
         <v>2742</v>
       </c>
@@ -15822,7 +15822,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="237" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="237" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A237">
         <v>2743</v>
       </c>
@@ -15887,7 +15887,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="238" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="238" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A238">
         <v>2744</v>
       </c>
@@ -15952,7 +15952,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="239" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="239" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A239">
         <v>2745</v>
       </c>
@@ -16017,7 +16017,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="240" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="240" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A240">
         <v>2746</v>
       </c>
@@ -16082,7 +16082,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="241" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="241" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A241">
         <v>2747</v>
       </c>
@@ -16147,7 +16147,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="242" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="242" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A242">
         <v>2748</v>
       </c>
@@ -16212,7 +16212,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="243" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="243" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A243">
         <v>2749</v>
       </c>
@@ -16277,7 +16277,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="244" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="244" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A244">
         <v>2750</v>
       </c>
@@ -16342,7 +16342,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="245" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="245" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A245">
         <v>2751</v>
       </c>
@@ -16407,7 +16407,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="246" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="246" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A246">
         <v>2752</v>
       </c>
@@ -16472,7 +16472,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="247" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="247" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A247">
         <v>2753</v>
       </c>
@@ -16537,7 +16537,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="248" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="248" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A248">
         <v>2754</v>
       </c>
@@ -16602,7 +16602,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="249" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="249" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A249">
         <v>2755</v>
       </c>
@@ -16667,7 +16667,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="250" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="250" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A250">
         <v>2756</v>
       </c>
@@ -16732,7 +16732,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="251" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="251" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A251">
         <v>2757</v>
       </c>
@@ -16797,7 +16797,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="252" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="252" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A252">
         <v>2758</v>
       </c>
@@ -16862,7 +16862,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="253" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="253" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A253">
         <v>2759</v>
       </c>
@@ -16927,7 +16927,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="254" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="254" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A254">
         <v>2760</v>
       </c>
@@ -16992,7 +16992,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="255" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="255" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A255">
         <v>2761</v>
       </c>
@@ -17057,7 +17057,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="256" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="256" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A256">
         <v>2762</v>
       </c>
@@ -17122,7 +17122,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="257" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="257" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A257">
         <v>2763</v>
       </c>
@@ -17187,7 +17187,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="258" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="258" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A258">
         <v>2764</v>
       </c>
@@ -17252,7 +17252,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="259" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="259" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A259">
         <v>2765</v>
       </c>
@@ -17317,7 +17317,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="260" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="260" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A260">
         <v>2766</v>
       </c>
@@ -17382,7 +17382,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="261" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="261" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A261">
         <v>2767</v>
       </c>
@@ -17447,7 +17447,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="262" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="262" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A262">
         <v>2768</v>
       </c>
@@ -17512,7 +17512,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="263" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="263" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A263">
         <v>2769</v>
       </c>
@@ -17577,7 +17577,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="264" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="264" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A264">
         <v>2770</v>
       </c>
@@ -17642,7 +17642,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="265" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="265" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A265">
         <v>2771</v>
       </c>
@@ -17707,7 +17707,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="266" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="266" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A266">
         <v>2772</v>
       </c>
@@ -17772,7 +17772,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="267" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="267" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A267">
         <v>2773</v>
       </c>
@@ -17837,7 +17837,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="268" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="268" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A268">
         <v>2774</v>
       </c>
@@ -17902,7 +17902,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="269" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="269" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A269">
         <v>2775</v>
       </c>
@@ -17967,7 +17967,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="270" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="270" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A270">
         <v>2776</v>
       </c>
@@ -18032,7 +18032,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="271" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="271" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A271">
         <v>2777</v>
       </c>
@@ -18097,7 +18097,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="272" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="272" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A272">
         <v>2778</v>
       </c>
@@ -18162,7 +18162,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="273" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="273" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A273">
         <v>2779</v>
       </c>
@@ -18227,7 +18227,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="274" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="274" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A274">
         <v>2780</v>
       </c>
@@ -18292,7 +18292,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="275" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="275" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A275">
         <v>2781</v>
       </c>
@@ -18357,7 +18357,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="276" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="276" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A276">
         <v>2782</v>
       </c>
@@ -18422,7 +18422,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="277" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="277" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A277">
         <v>2783</v>
       </c>
@@ -18487,7 +18487,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="278" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="278" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A278">
         <v>2784</v>
       </c>
@@ -18552,7 +18552,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="279" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="279" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A279">
         <v>2785</v>
       </c>
@@ -18617,7 +18617,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="280" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="280" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A280">
         <v>2786</v>
       </c>
@@ -18682,7 +18682,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="281" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="281" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A281">
         <v>2787</v>
       </c>
@@ -18747,7 +18747,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="282" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="282" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A282">
         <v>2788</v>
       </c>
@@ -18812,7 +18812,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="283" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="283" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A283">
         <v>2789</v>
       </c>
@@ -18877,7 +18877,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="284" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="284" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A284">
         <v>2790</v>
       </c>
@@ -18942,7 +18942,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="285" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="285" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A285">
         <v>2791</v>
       </c>
@@ -19007,7 +19007,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="286" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="286" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A286">
         <v>2792</v>
       </c>
@@ -19072,7 +19072,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="287" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="287" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A287">
         <v>2793</v>
       </c>
@@ -19137,7 +19137,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="288" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="288" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A288">
         <v>2794</v>
       </c>
@@ -19202,7 +19202,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="289" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="289" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A289">
         <v>2795</v>
       </c>
@@ -19267,7 +19267,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="290" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="290" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A290">
         <v>2796</v>
       </c>
@@ -19332,7 +19332,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="291" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="291" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A291">
         <v>2797</v>
       </c>
@@ -19397,7 +19397,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="292" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="292" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A292">
         <v>2798</v>
       </c>
@@ -19462,7 +19462,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="293" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="293" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A293">
         <v>2799</v>
       </c>
@@ -19527,7 +19527,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="294" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="294" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A294">
         <v>2800</v>
       </c>
@@ -19592,7 +19592,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="295" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="295" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A295">
         <v>2801</v>
       </c>
@@ -19657,7 +19657,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="296" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="296" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A296">
         <v>2802</v>
       </c>
@@ -19722,7 +19722,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="297" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="297" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A297">
         <v>2803</v>
       </c>
@@ -19787,7 +19787,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="298" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="298" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A298">
         <v>2804</v>
       </c>
@@ -19852,7 +19852,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="299" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="299" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A299">
         <v>2805</v>
       </c>
@@ -19917,7 +19917,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="300" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="300" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A300">
         <v>2806</v>
       </c>
@@ -19982,7 +19982,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="301" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="301" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A301">
         <v>2807</v>
       </c>
@@ -20047,7 +20047,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="302" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="302" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A302">
         <v>2808</v>
       </c>
@@ -20112,7 +20112,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="303" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="303" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A303">
         <v>2809</v>
       </c>
@@ -20177,7 +20177,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="304" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="304" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A304">
         <v>2810</v>
       </c>
@@ -20242,7 +20242,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="305" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="305" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A305">
         <v>2811</v>
       </c>
@@ -20307,7 +20307,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="306" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="306" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A306">
         <v>2812</v>
       </c>
@@ -20372,7 +20372,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="307" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="307" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A307">
         <v>2813</v>
       </c>
@@ -20437,7 +20437,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="308" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="308" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A308">
         <v>2814</v>
       </c>
@@ -20502,7 +20502,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="309" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="309" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A309">
         <v>2815</v>
       </c>
@@ -20567,7 +20567,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="310" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="310" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A310">
         <v>2816</v>
       </c>
@@ -20632,7 +20632,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="311" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="311" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A311">
         <v>2817</v>
       </c>
@@ -20697,7 +20697,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="312" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="312" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A312">
         <v>2818</v>
       </c>
@@ -20762,7 +20762,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="313" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="313" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A313">
         <v>2819</v>
       </c>
@@ -20827,7 +20827,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="314" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="314" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A314">
         <v>2820</v>
       </c>
@@ -20892,7 +20892,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="315" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="315" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A315">
         <v>2821</v>
       </c>
@@ -20957,7 +20957,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="316" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="316" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A316">
         <v>2822</v>
       </c>
@@ -21022,7 +21022,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="317" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="317" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A317">
         <v>2823</v>
       </c>
@@ -21087,7 +21087,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="318" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="318" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A318">
         <v>2824</v>
       </c>
@@ -21152,7 +21152,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="319" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="319" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A319">
         <v>2825</v>
       </c>
@@ -21217,7 +21217,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="320" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="320" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A320">
         <v>2826</v>
       </c>
@@ -21282,7 +21282,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="321" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="321" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A321">
         <v>2827</v>
       </c>
@@ -21347,7 +21347,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="322" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="322" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A322">
         <v>2828</v>
       </c>
@@ -21412,7 +21412,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="323" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="323" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A323">
         <v>2829</v>
       </c>
@@ -21477,7 +21477,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="324" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="324" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A324">
         <v>2830</v>
       </c>
@@ -21542,7 +21542,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="325" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="325" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A325">
         <v>2831</v>
       </c>
@@ -21607,7 +21607,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="326" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="326" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A326">
         <v>2832</v>
       </c>
@@ -21672,7 +21672,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="327" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="327" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A327">
         <v>2833</v>
       </c>
@@ -21737,7 +21737,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="328" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="328" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A328">
         <v>2834</v>
       </c>
@@ -21802,7 +21802,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="329" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="329" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A329">
         <v>2835</v>
       </c>
@@ -21867,7 +21867,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="330" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="330" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A330">
         <v>2836</v>
       </c>
@@ -21932,7 +21932,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="331" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="331" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A331">
         <v>2837</v>
       </c>
@@ -21997,7 +21997,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="332" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="332" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A332">
         <v>2838</v>
       </c>
@@ -22062,7 +22062,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="333" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="333" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A333">
         <v>2839</v>
       </c>
@@ -22127,7 +22127,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="334" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="334" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A334">
         <v>2840</v>
       </c>
@@ -22192,7 +22192,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="335" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="335" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A335">
         <v>2841</v>
       </c>
@@ -22257,7 +22257,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="336" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="336" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A336">
         <v>2842</v>
       </c>
@@ -22322,7 +22322,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="337" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="337" spans="1:22" x14ac:dyDescent="0.45">
       <c r="A337">
         <v>2843</v>
       </c>
@@ -22387,7 +22387,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="338" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="338" spans="1:22" x14ac:dyDescent="0.45">
       <c r="A338">
         <v>2844</v>
       </c>
@@ -22452,7 +22452,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="339" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="339" spans="1:22" x14ac:dyDescent="0.45">
       <c r="A339">
         <v>2845</v>
       </c>
@@ -22517,7 +22517,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="340" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="340" spans="1:22" x14ac:dyDescent="0.45">
       <c r="A340">
         <v>2846</v>
       </c>
@@ -22582,7 +22582,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="341" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="341" spans="1:22" x14ac:dyDescent="0.45">
       <c r="A341">
         <v>2847</v>
       </c>
@@ -22647,7 +22647,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="342" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="342" spans="1:22" x14ac:dyDescent="0.45">
       <c r="A342">
         <v>2848</v>
       </c>
@@ -22712,7 +22712,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="343" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="343" spans="1:22" x14ac:dyDescent="0.45">
       <c r="A343">
         <v>2848</v>
       </c>
@@ -22780,7 +22780,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="344" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="344" spans="1:22" x14ac:dyDescent="0.45">
       <c r="A344">
         <v>2850</v>
       </c>
@@ -22845,7 +22845,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="345" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="345" spans="1:22" x14ac:dyDescent="0.45">
       <c r="A345">
         <v>2851</v>
       </c>
@@ -22910,7 +22910,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="346" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="346" spans="1:22" x14ac:dyDescent="0.45">
       <c r="A346">
         <v>2852</v>
       </c>
@@ -22975,7 +22975,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="347" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="347" spans="1:22" x14ac:dyDescent="0.45">
       <c r="A347">
         <v>2853</v>
       </c>
@@ -23040,7 +23040,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="348" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="348" spans="1:22" x14ac:dyDescent="0.45">
       <c r="A348">
         <v>2854</v>
       </c>
@@ -23105,7 +23105,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="349" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="349" spans="1:22" x14ac:dyDescent="0.45">
       <c r="A349">
         <v>2855</v>
       </c>
@@ -23170,7 +23170,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="350" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="350" spans="1:22" x14ac:dyDescent="0.45">
       <c r="A350">
         <v>2856</v>
       </c>
@@ -23235,7 +23235,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="351" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="351" spans="1:22" x14ac:dyDescent="0.45">
       <c r="A351">
         <v>2857</v>
       </c>
@@ -23300,7 +23300,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="352" spans="1:22" x14ac:dyDescent="0.4">
+    <row r="352" spans="1:22" x14ac:dyDescent="0.45">
       <c r="A352">
         <v>2858</v>
       </c>
@@ -23365,7 +23365,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="353" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="353" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A353">
         <v>2859</v>
       </c>
@@ -23430,7 +23430,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="354" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="354" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A354">
         <v>2860</v>
       </c>
@@ -23495,7 +23495,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="355" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="355" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A355">
         <v>2861</v>
       </c>
@@ -23560,7 +23560,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="356" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="356" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A356">
         <v>2862</v>
       </c>
@@ -23625,7 +23625,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="357" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="357" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A357">
         <v>2863</v>
       </c>
@@ -23690,7 +23690,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="358" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="358" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A358">
         <v>2864</v>
       </c>
@@ -23755,7 +23755,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="359" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="359" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A359">
         <v>2865</v>
       </c>
@@ -23820,7 +23820,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="360" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="360" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A360">
         <v>2866</v>
       </c>
@@ -23885,7 +23885,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="361" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="361" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A361">
         <v>2867</v>
       </c>
@@ -23950,7 +23950,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="362" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="362" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A362">
         <v>2868</v>
       </c>
@@ -24015,7 +24015,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="363" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="363" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A363">
         <v>2869</v>
       </c>
@@ -24080,7 +24080,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="364" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="364" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A364">
         <v>2870</v>
       </c>
@@ -24145,7 +24145,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="365" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="365" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A365">
         <v>2871</v>
       </c>
@@ -24210,7 +24210,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="366" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="366" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A366">
         <v>2872</v>
       </c>
@@ -24275,7 +24275,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="367" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="367" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A367">
         <v>2873</v>
       </c>
@@ -24340,7 +24340,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="368" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="368" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A368">
         <v>2874</v>
       </c>
@@ -24405,7 +24405,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="369" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="369" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A369">
         <v>2875</v>
       </c>
@@ -24470,7 +24470,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="370" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="370" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A370">
         <v>2876</v>
       </c>
@@ -24535,7 +24535,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="371" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="371" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A371">
         <v>2877</v>
       </c>
@@ -24600,7 +24600,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="372" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="372" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A372">
         <v>2878</v>
       </c>
@@ -24665,7 +24665,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="373" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="373" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A373">
         <v>2879</v>
       </c>
@@ -24730,7 +24730,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="374" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="374" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A374">
         <v>2880</v>
       </c>
@@ -24795,7 +24795,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="375" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="375" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A375">
         <v>2881</v>
       </c>
@@ -24860,7 +24860,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="376" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="376" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A376">
         <v>2882</v>
       </c>
@@ -24925,7 +24925,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="377" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="377" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A377">
         <v>2883</v>
       </c>
@@ -24990,7 +24990,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="378" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="378" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A378">
         <v>2884</v>
       </c>
@@ -25055,7 +25055,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="379" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="379" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A379">
         <v>2885</v>
       </c>
@@ -25120,7 +25120,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="380" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="380" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A380">
         <v>2886</v>
       </c>
@@ -25185,7 +25185,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="381" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="381" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A381">
         <v>2887</v>
       </c>
@@ -25250,7 +25250,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="382" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="382" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A382">
         <v>2888</v>
       </c>
@@ -25315,7 +25315,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="383" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="383" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A383">
         <v>2889</v>
       </c>
@@ -25380,7 +25380,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="384" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="384" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A384">
         <v>2890</v>
       </c>
@@ -25445,7 +25445,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="385" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="385" spans="1:21" x14ac:dyDescent="0.45">
       <c r="A385">
         <v>2891</v>
       </c>
@@ -25508,6 +25508,1046 @@
       </c>
       <c r="U385">
         <v>97</v>
+      </c>
+    </row>
+    <row r="386" spans="1:21" x14ac:dyDescent="0.45">
+      <c r="A386">
+        <v>2892</v>
+      </c>
+      <c r="B386">
+        <v>9</v>
+      </c>
+      <c r="C386">
+        <v>13</v>
+      </c>
+      <c r="D386">
+        <v>28</v>
+      </c>
+      <c r="E386">
+        <v>32</v>
+      </c>
+      <c r="F386">
+        <v>40</v>
+      </c>
+      <c r="G386">
+        <v>42</v>
+      </c>
+      <c r="H386">
+        <v>45</v>
+      </c>
+      <c r="I386">
+        <v>48</v>
+      </c>
+      <c r="J386">
+        <v>57</v>
+      </c>
+      <c r="K386">
+        <v>59</v>
+      </c>
+      <c r="L386">
+        <v>61</v>
+      </c>
+      <c r="M386">
+        <v>64</v>
+      </c>
+      <c r="N386">
+        <v>66</v>
+      </c>
+      <c r="O386">
+        <v>70</v>
+      </c>
+      <c r="P386">
+        <v>75</v>
+      </c>
+      <c r="Q386">
+        <v>76</v>
+      </c>
+      <c r="R386">
+        <v>77</v>
+      </c>
+      <c r="S386">
+        <v>78</v>
+      </c>
+      <c r="T386">
+        <v>80</v>
+      </c>
+      <c r="U386">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="387" spans="1:21" x14ac:dyDescent="0.45">
+      <c r="A387">
+        <v>2893</v>
+      </c>
+      <c r="B387">
+        <v>0</v>
+      </c>
+      <c r="C387">
+        <v>2</v>
+      </c>
+      <c r="D387">
+        <v>5</v>
+      </c>
+      <c r="E387">
+        <v>6</v>
+      </c>
+      <c r="F387">
+        <v>16</v>
+      </c>
+      <c r="G387">
+        <v>23</v>
+      </c>
+      <c r="H387">
+        <v>29</v>
+      </c>
+      <c r="I387">
+        <v>32</v>
+      </c>
+      <c r="J387">
+        <v>39</v>
+      </c>
+      <c r="K387">
+        <v>43</v>
+      </c>
+      <c r="L387">
+        <v>44</v>
+      </c>
+      <c r="M387">
+        <v>51</v>
+      </c>
+      <c r="N387">
+        <v>53</v>
+      </c>
+      <c r="O387">
+        <v>61</v>
+      </c>
+      <c r="P387">
+        <v>67</v>
+      </c>
+      <c r="Q387">
+        <v>68</v>
+      </c>
+      <c r="R387">
+        <v>89</v>
+      </c>
+      <c r="S387">
+        <v>93</v>
+      </c>
+      <c r="T387">
+        <v>98</v>
+      </c>
+      <c r="U387">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="388" spans="1:21" x14ac:dyDescent="0.45">
+      <c r="A388">
+        <v>2894</v>
+      </c>
+      <c r="B388">
+        <v>4</v>
+      </c>
+      <c r="C388">
+        <v>6</v>
+      </c>
+      <c r="D388">
+        <v>12</v>
+      </c>
+      <c r="E388">
+        <v>15</v>
+      </c>
+      <c r="F388">
+        <v>17</v>
+      </c>
+      <c r="G388">
+        <v>19</v>
+      </c>
+      <c r="H388">
+        <v>24</v>
+      </c>
+      <c r="I388">
+        <v>27</v>
+      </c>
+      <c r="J388">
+        <v>32</v>
+      </c>
+      <c r="K388">
+        <v>38</v>
+      </c>
+      <c r="L388">
+        <v>40</v>
+      </c>
+      <c r="M388">
+        <v>47</v>
+      </c>
+      <c r="N388">
+        <v>52</v>
+      </c>
+      <c r="O388">
+        <v>63</v>
+      </c>
+      <c r="P388">
+        <v>71</v>
+      </c>
+      <c r="Q388">
+        <v>74</v>
+      </c>
+      <c r="R388">
+        <v>75</v>
+      </c>
+      <c r="S388">
+        <v>78</v>
+      </c>
+      <c r="T388">
+        <v>80</v>
+      </c>
+      <c r="U388">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="389" spans="1:21" x14ac:dyDescent="0.45">
+      <c r="A389">
+        <v>2895</v>
+      </c>
+      <c r="B389">
+        <v>1</v>
+      </c>
+      <c r="C389">
+        <v>16</v>
+      </c>
+      <c r="D389">
+        <v>22</v>
+      </c>
+      <c r="E389">
+        <v>23</v>
+      </c>
+      <c r="F389">
+        <v>27</v>
+      </c>
+      <c r="G389">
+        <v>29</v>
+      </c>
+      <c r="H389">
+        <v>30</v>
+      </c>
+      <c r="I389">
+        <v>32</v>
+      </c>
+      <c r="J389">
+        <v>42</v>
+      </c>
+      <c r="K389">
+        <v>44</v>
+      </c>
+      <c r="L389">
+        <v>45</v>
+      </c>
+      <c r="M389">
+        <v>55</v>
+      </c>
+      <c r="N389">
+        <v>58</v>
+      </c>
+      <c r="O389">
+        <v>66</v>
+      </c>
+      <c r="P389">
+        <v>79</v>
+      </c>
+      <c r="Q389">
+        <v>88</v>
+      </c>
+      <c r="R389">
+        <v>89</v>
+      </c>
+      <c r="S389">
+        <v>90</v>
+      </c>
+      <c r="T389">
+        <v>91</v>
+      </c>
+      <c r="U389">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="390" spans="1:21" x14ac:dyDescent="0.45">
+      <c r="A390">
+        <v>2896</v>
+      </c>
+      <c r="B390">
+        <v>9</v>
+      </c>
+      <c r="C390">
+        <v>11</v>
+      </c>
+      <c r="D390">
+        <v>12</v>
+      </c>
+      <c r="E390">
+        <v>13</v>
+      </c>
+      <c r="F390">
+        <v>24</v>
+      </c>
+      <c r="G390">
+        <v>25</v>
+      </c>
+      <c r="H390">
+        <v>26</v>
+      </c>
+      <c r="I390">
+        <v>28</v>
+      </c>
+      <c r="J390">
+        <v>31</v>
+      </c>
+      <c r="K390">
+        <v>34</v>
+      </c>
+      <c r="L390">
+        <v>36</v>
+      </c>
+      <c r="M390">
+        <v>39</v>
+      </c>
+      <c r="N390">
+        <v>42</v>
+      </c>
+      <c r="O390">
+        <v>43</v>
+      </c>
+      <c r="P390">
+        <v>53</v>
+      </c>
+      <c r="Q390">
+        <v>75</v>
+      </c>
+      <c r="R390">
+        <v>76</v>
+      </c>
+      <c r="S390">
+        <v>78</v>
+      </c>
+      <c r="T390">
+        <v>83</v>
+      </c>
+      <c r="U390">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="391" spans="1:21" x14ac:dyDescent="0.45">
+      <c r="A391">
+        <v>2897</v>
+      </c>
+      <c r="B391">
+        <v>9</v>
+      </c>
+      <c r="C391">
+        <v>11</v>
+      </c>
+      <c r="D391">
+        <v>19</v>
+      </c>
+      <c r="E391">
+        <v>24</v>
+      </c>
+      <c r="F391">
+        <v>25</v>
+      </c>
+      <c r="G391">
+        <v>31</v>
+      </c>
+      <c r="H391">
+        <v>38</v>
+      </c>
+      <c r="I391">
+        <v>43</v>
+      </c>
+      <c r="J391">
+        <v>46</v>
+      </c>
+      <c r="K391">
+        <v>47</v>
+      </c>
+      <c r="L391">
+        <v>48</v>
+      </c>
+      <c r="M391">
+        <v>66</v>
+      </c>
+      <c r="N391">
+        <v>69</v>
+      </c>
+      <c r="O391">
+        <v>70</v>
+      </c>
+      <c r="P391">
+        <v>73</v>
+      </c>
+      <c r="Q391">
+        <v>83</v>
+      </c>
+      <c r="R391">
+        <v>84</v>
+      </c>
+      <c r="S391">
+        <v>88</v>
+      </c>
+      <c r="T391">
+        <v>90</v>
+      </c>
+      <c r="U391">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="392" spans="1:21" x14ac:dyDescent="0.45">
+      <c r="A392">
+        <v>2898</v>
+      </c>
+      <c r="B392">
+        <v>0</v>
+      </c>
+      <c r="C392">
+        <v>2</v>
+      </c>
+      <c r="D392">
+        <v>4</v>
+      </c>
+      <c r="E392">
+        <v>6</v>
+      </c>
+      <c r="F392">
+        <v>11</v>
+      </c>
+      <c r="G392">
+        <v>15</v>
+      </c>
+      <c r="H392">
+        <v>20</v>
+      </c>
+      <c r="I392">
+        <v>28</v>
+      </c>
+      <c r="J392">
+        <v>37</v>
+      </c>
+      <c r="K392">
+        <v>39</v>
+      </c>
+      <c r="L392">
+        <v>45</v>
+      </c>
+      <c r="M392">
+        <v>51</v>
+      </c>
+      <c r="N392">
+        <v>52</v>
+      </c>
+      <c r="O392">
+        <v>53</v>
+      </c>
+      <c r="P392">
+        <v>59</v>
+      </c>
+      <c r="Q392">
+        <v>62</v>
+      </c>
+      <c r="R392">
+        <v>73</v>
+      </c>
+      <c r="S392">
+        <v>75</v>
+      </c>
+      <c r="T392">
+        <v>79</v>
+      </c>
+      <c r="U392">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="393" spans="1:21" x14ac:dyDescent="0.45">
+      <c r="A393">
+        <v>2899</v>
+      </c>
+      <c r="B393">
+        <v>23</v>
+      </c>
+      <c r="C393">
+        <v>26</v>
+      </c>
+      <c r="D393">
+        <v>27</v>
+      </c>
+      <c r="E393">
+        <v>29</v>
+      </c>
+      <c r="F393">
+        <v>31</v>
+      </c>
+      <c r="G393">
+        <v>37</v>
+      </c>
+      <c r="H393">
+        <v>49</v>
+      </c>
+      <c r="I393">
+        <v>52</v>
+      </c>
+      <c r="J393">
+        <v>55</v>
+      </c>
+      <c r="K393">
+        <v>58</v>
+      </c>
+      <c r="L393">
+        <v>61</v>
+      </c>
+      <c r="M393">
+        <v>71</v>
+      </c>
+      <c r="N393">
+        <v>74</v>
+      </c>
+      <c r="O393">
+        <v>79</v>
+      </c>
+      <c r="P393">
+        <v>82</v>
+      </c>
+      <c r="Q393">
+        <v>88</v>
+      </c>
+      <c r="R393">
+        <v>89</v>
+      </c>
+      <c r="S393">
+        <v>95</v>
+      </c>
+      <c r="T393">
+        <v>96</v>
+      </c>
+      <c r="U393">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="394" spans="1:21" x14ac:dyDescent="0.45">
+      <c r="A394">
+        <v>2900</v>
+      </c>
+      <c r="B394">
+        <v>4</v>
+      </c>
+      <c r="C394">
+        <v>11</v>
+      </c>
+      <c r="D394">
+        <v>14</v>
+      </c>
+      <c r="E394">
+        <v>26</v>
+      </c>
+      <c r="F394">
+        <v>27</v>
+      </c>
+      <c r="G394">
+        <v>29</v>
+      </c>
+      <c r="H394">
+        <v>30</v>
+      </c>
+      <c r="I394">
+        <v>35</v>
+      </c>
+      <c r="J394">
+        <v>40</v>
+      </c>
+      <c r="K394">
+        <v>41</v>
+      </c>
+      <c r="L394">
+        <v>43</v>
+      </c>
+      <c r="M394">
+        <v>58</v>
+      </c>
+      <c r="N394">
+        <v>62</v>
+      </c>
+      <c r="O394">
+        <v>64</v>
+      </c>
+      <c r="P394">
+        <v>83</v>
+      </c>
+      <c r="Q394">
+        <v>90</v>
+      </c>
+      <c r="R394">
+        <v>92</v>
+      </c>
+      <c r="S394">
+        <v>95</v>
+      </c>
+      <c r="T394">
+        <v>96</v>
+      </c>
+      <c r="U394">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="395" spans="1:21" x14ac:dyDescent="0.45">
+      <c r="A395">
+        <v>2901</v>
+      </c>
+      <c r="B395">
+        <v>5</v>
+      </c>
+      <c r="C395">
+        <v>6</v>
+      </c>
+      <c r="D395">
+        <v>9</v>
+      </c>
+      <c r="E395">
+        <v>12</v>
+      </c>
+      <c r="F395">
+        <v>13</v>
+      </c>
+      <c r="G395">
+        <v>16</v>
+      </c>
+      <c r="H395">
+        <v>25</v>
+      </c>
+      <c r="I395">
+        <v>35</v>
+      </c>
+      <c r="J395">
+        <v>37</v>
+      </c>
+      <c r="K395">
+        <v>38</v>
+      </c>
+      <c r="L395">
+        <v>44</v>
+      </c>
+      <c r="M395">
+        <v>45</v>
+      </c>
+      <c r="N395">
+        <v>54</v>
+      </c>
+      <c r="O395">
+        <v>61</v>
+      </c>
+      <c r="P395">
+        <v>62</v>
+      </c>
+      <c r="Q395">
+        <v>69</v>
+      </c>
+      <c r="R395">
+        <v>73</v>
+      </c>
+      <c r="S395">
+        <v>79</v>
+      </c>
+      <c r="T395">
+        <v>95</v>
+      </c>
+      <c r="U395">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="396" spans="1:21" x14ac:dyDescent="0.45">
+      <c r="A396">
+        <v>2902</v>
+      </c>
+      <c r="B396">
+        <v>5</v>
+      </c>
+      <c r="C396">
+        <v>12</v>
+      </c>
+      <c r="D396">
+        <v>21</v>
+      </c>
+      <c r="E396">
+        <v>25</v>
+      </c>
+      <c r="F396">
+        <v>29</v>
+      </c>
+      <c r="G396">
+        <v>31</v>
+      </c>
+      <c r="H396">
+        <v>33</v>
+      </c>
+      <c r="I396">
+        <v>36</v>
+      </c>
+      <c r="J396">
+        <v>46</v>
+      </c>
+      <c r="K396">
+        <v>47</v>
+      </c>
+      <c r="L396">
+        <v>50</v>
+      </c>
+      <c r="M396">
+        <v>54</v>
+      </c>
+      <c r="N396">
+        <v>58</v>
+      </c>
+      <c r="O396">
+        <v>60</v>
+      </c>
+      <c r="P396">
+        <v>61</v>
+      </c>
+      <c r="Q396">
+        <v>66</v>
+      </c>
+      <c r="R396">
+        <v>68</v>
+      </c>
+      <c r="S396">
+        <v>72</v>
+      </c>
+      <c r="T396">
+        <v>78</v>
+      </c>
+      <c r="U396">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="397" spans="1:21" x14ac:dyDescent="0.45">
+      <c r="A397">
+        <v>2903</v>
+      </c>
+      <c r="B397">
+        <v>10</v>
+      </c>
+      <c r="C397">
+        <v>12</v>
+      </c>
+      <c r="D397">
+        <v>18</v>
+      </c>
+      <c r="E397">
+        <v>24</v>
+      </c>
+      <c r="F397">
+        <v>37</v>
+      </c>
+      <c r="G397">
+        <v>43</v>
+      </c>
+      <c r="H397">
+        <v>45</v>
+      </c>
+      <c r="I397">
+        <v>49</v>
+      </c>
+      <c r="J397">
+        <v>50</v>
+      </c>
+      <c r="K397">
+        <v>53</v>
+      </c>
+      <c r="L397">
+        <v>54</v>
+      </c>
+      <c r="M397">
+        <v>61</v>
+      </c>
+      <c r="N397">
+        <v>70</v>
+      </c>
+      <c r="O397">
+        <v>72</v>
+      </c>
+      <c r="P397">
+        <v>75</v>
+      </c>
+      <c r="Q397">
+        <v>82</v>
+      </c>
+      <c r="R397">
+        <v>89</v>
+      </c>
+      <c r="S397">
+        <v>93</v>
+      </c>
+      <c r="T397">
+        <v>95</v>
+      </c>
+      <c r="U397">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="398" spans="1:21" x14ac:dyDescent="0.45">
+      <c r="A398">
+        <v>2904</v>
+      </c>
+      <c r="B398">
+        <v>9</v>
+      </c>
+      <c r="C398">
+        <v>22</v>
+      </c>
+      <c r="D398">
+        <v>41</v>
+      </c>
+      <c r="E398">
+        <v>43</v>
+      </c>
+      <c r="F398">
+        <v>44</v>
+      </c>
+      <c r="G398">
+        <v>45</v>
+      </c>
+      <c r="H398">
+        <v>52</v>
+      </c>
+      <c r="I398">
+        <v>55</v>
+      </c>
+      <c r="J398">
+        <v>57</v>
+      </c>
+      <c r="K398">
+        <v>62</v>
+      </c>
+      <c r="L398">
+        <v>69</v>
+      </c>
+      <c r="M398">
+        <v>72</v>
+      </c>
+      <c r="N398">
+        <v>75</v>
+      </c>
+      <c r="O398">
+        <v>77</v>
+      </c>
+      <c r="P398">
+        <v>79</v>
+      </c>
+      <c r="Q398">
+        <v>87</v>
+      </c>
+      <c r="R398">
+        <v>91</v>
+      </c>
+      <c r="S398">
+        <v>93</v>
+      </c>
+      <c r="T398">
+        <v>96</v>
+      </c>
+      <c r="U398">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="399" spans="1:21" x14ac:dyDescent="0.45">
+      <c r="A399">
+        <v>2905</v>
+      </c>
+      <c r="B399">
+        <v>6</v>
+      </c>
+      <c r="C399">
+        <v>7</v>
+      </c>
+      <c r="D399">
+        <v>9</v>
+      </c>
+      <c r="E399">
+        <v>14</v>
+      </c>
+      <c r="F399">
+        <v>17</v>
+      </c>
+      <c r="G399">
+        <v>22</v>
+      </c>
+      <c r="H399">
+        <v>29</v>
+      </c>
+      <c r="I399">
+        <v>32</v>
+      </c>
+      <c r="J399">
+        <v>36</v>
+      </c>
+      <c r="K399">
+        <v>40</v>
+      </c>
+      <c r="L399">
+        <v>52</v>
+      </c>
+      <c r="M399">
+        <v>54</v>
+      </c>
+      <c r="N399">
+        <v>55</v>
+      </c>
+      <c r="O399">
+        <v>67</v>
+      </c>
+      <c r="P399">
+        <v>69</v>
+      </c>
+      <c r="Q399">
+        <v>73</v>
+      </c>
+      <c r="R399">
+        <v>74</v>
+      </c>
+      <c r="S399">
+        <v>78</v>
+      </c>
+      <c r="T399">
+        <v>91</v>
+      </c>
+      <c r="U399">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="400" spans="1:21" x14ac:dyDescent="0.45">
+      <c r="A400">
+        <v>2906</v>
+      </c>
+      <c r="B400">
+        <v>0</v>
+      </c>
+      <c r="C400">
+        <v>2</v>
+      </c>
+      <c r="D400">
+        <v>4</v>
+      </c>
+      <c r="E400">
+        <v>6</v>
+      </c>
+      <c r="F400">
+        <v>10</v>
+      </c>
+      <c r="G400">
+        <v>11</v>
+      </c>
+      <c r="H400">
+        <v>12</v>
+      </c>
+      <c r="I400">
+        <v>19</v>
+      </c>
+      <c r="J400">
+        <v>26</v>
+      </c>
+      <c r="K400">
+        <v>31</v>
+      </c>
+      <c r="L400">
+        <v>37</v>
+      </c>
+      <c r="M400">
+        <v>43</v>
+      </c>
+      <c r="N400">
+        <v>45</v>
+      </c>
+      <c r="O400">
+        <v>54</v>
+      </c>
+      <c r="P400">
+        <v>73</v>
+      </c>
+      <c r="Q400">
+        <v>74</v>
+      </c>
+      <c r="R400">
+        <v>76</v>
+      </c>
+      <c r="S400">
+        <v>79</v>
+      </c>
+      <c r="T400">
+        <v>91</v>
+      </c>
+      <c r="U400">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="401" spans="1:21" x14ac:dyDescent="0.45">
+      <c r="A401">
+        <v>2907</v>
+      </c>
+      <c r="B401">
+        <v>0</v>
+      </c>
+      <c r="C401">
+        <v>1</v>
+      </c>
+      <c r="D401">
+        <v>4</v>
+      </c>
+      <c r="E401">
+        <v>5</v>
+      </c>
+      <c r="F401">
+        <v>9</v>
+      </c>
+      <c r="G401">
+        <v>25</v>
+      </c>
+      <c r="H401">
+        <v>27</v>
+      </c>
+      <c r="I401">
+        <v>28</v>
+      </c>
+      <c r="J401">
+        <v>34</v>
+      </c>
+      <c r="K401">
+        <v>36</v>
+      </c>
+      <c r="L401">
+        <v>53</v>
+      </c>
+      <c r="M401">
+        <v>58</v>
+      </c>
+      <c r="N401">
+        <v>67</v>
+      </c>
+      <c r="O401">
+        <v>69</v>
+      </c>
+      <c r="P401">
+        <v>72</v>
+      </c>
+      <c r="Q401">
+        <v>80</v>
+      </c>
+      <c r="R401">
+        <v>82</v>
+      </c>
+      <c r="S401">
+        <v>93</v>
+      </c>
+      <c r="T401">
+        <v>94</v>
+      </c>
+      <c r="U401">
+        <v>96</v>
       </c>
     </row>
   </sheetData>
@@ -25516,25 +26556,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <PublishingExpirationDate xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <PublishingStartDate xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <AtualizadoPeloTimerJobEm xmlns="4455b8ba-124f-46d5-aaaa-9813efd83d1e">2025-08-09T04:04:08+00:00</AtualizadoPeloTimerJobEm>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x010100C92CDE8829F3C7438DCCB0991C30EAAE" ma:contentTypeVersion="3" ma:contentTypeDescription="Crie um novo documento." ma:contentTypeScope="" ma:versionID="36cf41eecaf38ba1d849a0c8dd067090">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns1="http://schemas.microsoft.com/sharepoint/v3" xmlns:ns2="3e38fcf2-aa96-4a2c-865b-c3abba01ba51" xmlns:ns3="4455b8ba-124f-46d5-aaaa-9813efd83d1e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="023f68b2d27389a617bf935a3f0e17ad" ns1:_="" ns2:_="" ns3:_="">
     <xsd:import namespace="http://schemas.microsoft.com/sharepoint/v3"/>
@@ -25702,26 +26723,26 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1EF4B058-BA16-41FB-9728-59896EB3A3A3}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
-    <ds:schemaRef ds:uri="4455b8ba-124f-46d5-aaaa-9813efd83d1e"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5603705F-A6C5-47C9-9C54-F9F7DF9013C0}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <PublishingExpirationDate xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <PublishingStartDate xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <AtualizadoPeloTimerJobEm xmlns="4455b8ba-124f-46d5-aaaa-9813efd83d1e">2025-08-09T04:04:08+00:00</AtualizadoPeloTimerJobEm>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FDEE3BD0-E82A-45EA-BF5A-733EBB4C31D1}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -25739,4 +26760,23 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5603705F-A6C5-47C9-9C54-F9F7DF9013C0}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1EF4B058-BA16-41FB-9728-59896EB3A3A3}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
+    <ds:schemaRef ds:uri="4455b8ba-124f-46d5-aaaa-9813efd83d1e"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>